<commit_message>
betzel-hateena: all inner pages in the home's treatment; hero points, rearranged collage, centred strip; pushed, live QA 0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GFjDY7i3KpUg2KGwnZs5PT
</commit_message>
<xml_diff>
--- a/sites/betzel-hateena/SEO-QA-betzel-hateena.xlsx
+++ b/sites/betzel-hateena/SEO-QA-betzel-hateena.xlsx
@@ -962,7 +962,7 @@
       </c>
       <c r="E12" s="17" t="inlineStr">
         <is>
-          <t>54 images</t>
+          <t>52 images</t>
         </is>
       </c>
       <c r="F12" s="16" t="n"/>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="E24" s="17" t="inlineStr">
         <is>
-          <t>17 internal links, all &lt; 400</t>
+          <t>16 internal links, all &lt; 400</t>
         </is>
       </c>
       <c r="F24" s="20" t="n"/>

</xml_diff>